<commit_message>
Apply review-round fixes to the confirmation workbook
Strict dropdowns that reject typed values; "Discuss" coloured red and
counted as negative to match the legend; Items counts as live COUNTA
formulas; legend lists exact dropdown values; example row greyed and
marked not editable; header rows frozen on single-table reference
sheets; Meditron and voice-conflict notes added; minor width fix.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USyWZdFCwDpe3L4dpdaCcG
</commit_message>
<xml_diff>
--- a/docs/ATLAS_REVIEW_CONFIRMATION.xlsx
+++ b/docs/ATLAS_REVIEW_CONFIRMATION.xlsx
@@ -71,7 +71,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -103,6 +103,11 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -130,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,11 +161,14 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -652,7 +660,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Accepted / Yes / Pass</t>
+          <t>Accept recommendation / Accept / Yes / N/A / Pass</t>
         </is>
       </c>
     </row>
@@ -730,8 +738,9 @@
           <t>1 Decisions</t>
         </is>
       </c>
-      <c r="B21" s="12" t="n">
-        <v>14</v>
+      <c r="B21" s="12">
+        <f>COUNTA('1 Decisions'!$A$5:$A$18)</f>
+        <v/>
       </c>
       <c r="C21" s="12">
         <f>B21-G21</f>
@@ -750,7 +759,7 @@
         <v/>
       </c>
       <c r="G21" s="12">
-        <f>COUNTBLANK('1 Decisions'!$E$5:$E$18)+COUNTIF('1 Decisions'!$E$5:$E$18,"Not yet run")</f>
+        <f>COUNTBLANK('1 Decisions'!$E$5:$E$18)</f>
         <v/>
       </c>
     </row>
@@ -760,8 +769,9 @@
           <t>2 Resolutions</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n">
-        <v>20</v>
+      <c r="B22" s="12">
+        <f>COUNTA('2 Resolutions'!$A$5:$A$24)</f>
+        <v/>
       </c>
       <c r="C22" s="12">
         <f>B22-G22</f>
@@ -780,7 +790,7 @@
         <v/>
       </c>
       <c r="G22" s="12">
-        <f>COUNTBLANK('2 Resolutions'!$D$5:$D$24)+COUNTIF('2 Resolutions'!$D$5:$D$24,"Not yet run")</f>
+        <f>COUNTBLANK('2 Resolutions'!$D$5:$D$24)</f>
         <v/>
       </c>
     </row>
@@ -790,8 +800,9 @@
           <t>3 Risks</t>
         </is>
       </c>
-      <c r="B23" s="12" t="n">
-        <v>18</v>
+      <c r="B23" s="12">
+        <f>COUNTA('3 Risks'!$A$5:$A$22)</f>
+        <v/>
       </c>
       <c r="C23" s="12">
         <f>B23-G23</f>
@@ -810,7 +821,7 @@
         <v/>
       </c>
       <c r="G23" s="12">
-        <f>COUNTBLANK('3 Risks'!$F$5:$F$22)+COUNTIF('3 Risks'!$F$5:$F$22,"Not yet run")</f>
+        <f>COUNTBLANK('3 Risks'!$F$5:$F$22)</f>
         <v/>
       </c>
     </row>
@@ -820,8 +831,9 @@
           <t>4 Verification</t>
         </is>
       </c>
-      <c r="B24" s="12" t="n">
-        <v>18</v>
+      <c r="B24" s="12">
+        <f>COUNTA('4 Verification'!$A$5:$A$22)</f>
+        <v/>
       </c>
       <c r="C24" s="12">
         <f>B24-G24</f>
@@ -850,8 +862,9 @@
           <t>5 Checklist</t>
         </is>
       </c>
-      <c r="B25" s="12" t="n">
-        <v>14</v>
+      <c r="B25" s="12">
+        <f>COUNTA('5 Checklist'!$A$5:$A$18)</f>
+        <v/>
       </c>
       <c r="C25" s="12">
         <f>B25-G25</f>
@@ -870,7 +883,7 @@
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTBLANK('5 Checklist'!$D$5:$D$18)+COUNTIF('5 Checklist'!$D$5:$D$18,"Not yet run")</f>
+        <f>COUNTBLANK('5 Checklist'!$D$5:$D$18)</f>
         <v/>
       </c>
     </row>
@@ -915,7 +928,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Example of a completed decision row (format only; not a real answer)</t>
+          <t>Example of a completed decision row (format only, not editable, not counted; grey marks where your text would go)</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1672,6 +1685,13 @@
       <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Kokoro preset</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Known conflict: Arthur, Victor, and Gideon all pull toward the same four British male presets. Once heard, expect to spread them apart or move one to a Chatterbox clone, as Alaric is.</t>
         </is>
       </c>
     </row>
@@ -3315,8 +3335,8 @@
         </is>
       </c>
       <c r="E5" s="16" t="n"/>
-      <c r="F5" s="15" t="n"/>
-      <c r="G5" s="15" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -3340,8 +3360,8 @@
         </is>
       </c>
       <c r="E6" s="16" t="n"/>
-      <c r="F6" s="15" t="n"/>
-      <c r="G6" s="15" t="n"/>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -3365,8 +3385,8 @@
         </is>
       </c>
       <c r="E7" s="16" t="n"/>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="15" t="n"/>
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -3390,8 +3410,8 @@
         </is>
       </c>
       <c r="E8" s="16" t="n"/>
-      <c r="F8" s="15" t="n"/>
-      <c r="G8" s="15" t="n"/>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3415,8 +3435,8 @@
         </is>
       </c>
       <c r="E9" s="16" t="n"/>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="15" t="n"/>
+      <c r="F9" s="17" t="n"/>
+      <c r="G9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -3440,8 +3460,8 @@
         </is>
       </c>
       <c r="E10" s="16" t="n"/>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="15" t="n"/>
+      <c r="F10" s="17" t="n"/>
+      <c r="G10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3465,8 +3485,8 @@
         </is>
       </c>
       <c r="E11" s="16" t="n"/>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="15" t="n"/>
+      <c r="F11" s="17" t="n"/>
+      <c r="G11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -3490,8 +3510,8 @@
         </is>
       </c>
       <c r="E12" s="16" t="n"/>
-      <c r="F12" s="15" t="n"/>
-      <c r="G12" s="15" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -3515,8 +3535,8 @@
         </is>
       </c>
       <c r="E13" s="16" t="n"/>
-      <c r="F13" s="15" t="n"/>
-      <c r="G13" s="15" t="n"/>
+      <c r="F13" s="17" t="n"/>
+      <c r="G13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -3540,8 +3560,8 @@
         </is>
       </c>
       <c r="E14" s="16" t="n"/>
-      <c r="F14" s="15" t="n"/>
-      <c r="G14" s="15" t="n"/>
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -3565,8 +3585,8 @@
         </is>
       </c>
       <c r="E15" s="16" t="n"/>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -3590,8 +3610,8 @@
         </is>
       </c>
       <c r="E16" s="16" t="n"/>
-      <c r="F16" s="15" t="n"/>
-      <c r="G16" s="15" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -3615,8 +3635,8 @@
         </is>
       </c>
       <c r="E17" s="16" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
+      <c r="F17" s="17" t="n"/>
+      <c r="G17" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -3640,8 +3660,8 @@
         </is>
       </c>
       <c r="E18" s="16" t="n"/>
-      <c r="F18" s="15" t="n"/>
-      <c r="G18" s="15" t="n"/>
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="17" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:G18"/>
@@ -3657,7 +3677,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E5:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Accept recommendation / Change / Need more information" type="list">
+    <dataValidation sqref="E5:E18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Accept recommendation / Change / Need more information" type="list" errorStyle="stop">
       <formula1>"Accept recommendation,Change,Need more information"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3739,7 +3759,7 @@
         </is>
       </c>
       <c r="D5" s="16" t="n"/>
-      <c r="E5" s="15" t="n"/>
+      <c r="E5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -3758,7 +3778,7 @@
         </is>
       </c>
       <c r="D6" s="16" t="n"/>
-      <c r="E6" s="15" t="n"/>
+      <c r="E6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -3777,7 +3797,7 @@
         </is>
       </c>
       <c r="D7" s="16" t="n"/>
-      <c r="E7" s="15" t="n"/>
+      <c r="E7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -3796,7 +3816,7 @@
         </is>
       </c>
       <c r="D8" s="16" t="n"/>
-      <c r="E8" s="15" t="n"/>
+      <c r="E8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -3815,7 +3835,7 @@
         </is>
       </c>
       <c r="D9" s="16" t="n"/>
-      <c r="E9" s="15" t="n"/>
+      <c r="E9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -3834,7 +3854,7 @@
         </is>
       </c>
       <c r="D10" s="16" t="n"/>
-      <c r="E10" s="15" t="n"/>
+      <c r="E10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -3853,7 +3873,7 @@
         </is>
       </c>
       <c r="D11" s="16" t="n"/>
-      <c r="E11" s="15" t="n"/>
+      <c r="E11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -3872,7 +3892,7 @@
         </is>
       </c>
       <c r="D12" s="16" t="n"/>
-      <c r="E12" s="15" t="n"/>
+      <c r="E12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -3891,7 +3911,7 @@
         </is>
       </c>
       <c r="D13" s="16" t="n"/>
-      <c r="E13" s="15" t="n"/>
+      <c r="E13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -3910,7 +3930,7 @@
         </is>
       </c>
       <c r="D14" s="16" t="n"/>
-      <c r="E14" s="15" t="n"/>
+      <c r="E14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -3929,7 +3949,7 @@
         </is>
       </c>
       <c r="D15" s="16" t="n"/>
-      <c r="E15" s="15" t="n"/>
+      <c r="E15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -3948,7 +3968,7 @@
         </is>
       </c>
       <c r="D16" s="16" t="n"/>
-      <c r="E16" s="15" t="n"/>
+      <c r="E16" s="17" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -3967,7 +3987,7 @@
         </is>
       </c>
       <c r="D17" s="16" t="n"/>
-      <c r="E17" s="15" t="n"/>
+      <c r="E17" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -3986,7 +4006,7 @@
         </is>
       </c>
       <c r="D18" s="16" t="n"/>
-      <c r="E18" s="15" t="n"/>
+      <c r="E18" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -4005,7 +4025,7 @@
         </is>
       </c>
       <c r="D19" s="16" t="n"/>
-      <c r="E19" s="15" t="n"/>
+      <c r="E19" s="17" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -4024,7 +4044,7 @@
         </is>
       </c>
       <c r="D20" s="16" t="n"/>
-      <c r="E20" s="15" t="n"/>
+      <c r="E20" s="17" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -4043,7 +4063,7 @@
         </is>
       </c>
       <c r="D21" s="16" t="n"/>
-      <c r="E21" s="15" t="n"/>
+      <c r="E21" s="17" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
@@ -4062,7 +4082,7 @@
         </is>
       </c>
       <c r="D22" s="16" t="n"/>
-      <c r="E22" s="15" t="n"/>
+      <c r="E22" s="17" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
@@ -4081,7 +4101,7 @@
         </is>
       </c>
       <c r="D23" s="16" t="n"/>
-      <c r="E23" s="15" t="n"/>
+      <c r="E23" s="17" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
@@ -4100,7 +4120,7 @@
         </is>
       </c>
       <c r="D24" s="16" t="n"/>
-      <c r="E24" s="15" t="n"/>
+      <c r="E24" s="17" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:E24"/>
@@ -4113,7 +4133,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Accept / Disagree - return to decisions" type="list">
+    <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Accept / Disagree - return to decisions" type="list" errorStyle="stop">
       <formula1>"Accept,Disagree - return to decisions"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4217,7 +4237,7 @@
         </is>
       </c>
       <c r="F5" s="16" t="n"/>
-      <c r="G5" s="15" t="n"/>
+      <c r="G5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -4246,7 +4266,7 @@
         </is>
       </c>
       <c r="F6" s="16" t="n"/>
-      <c r="G6" s="15" t="n"/>
+      <c r="G6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -4275,7 +4295,7 @@
         </is>
       </c>
       <c r="F7" s="16" t="n"/>
-      <c r="G7" s="15" t="n"/>
+      <c r="G7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -4304,7 +4324,7 @@
         </is>
       </c>
       <c r="F8" s="16" t="n"/>
-      <c r="G8" s="15" t="n"/>
+      <c r="G8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4333,7 +4353,7 @@
         </is>
       </c>
       <c r="F9" s="16" t="n"/>
-      <c r="G9" s="15" t="n"/>
+      <c r="G9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -4362,7 +4382,7 @@
         </is>
       </c>
       <c r="F10" s="16" t="n"/>
-      <c r="G10" s="15" t="n"/>
+      <c r="G10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4391,7 +4411,7 @@
         </is>
       </c>
       <c r="F11" s="16" t="n"/>
-      <c r="G11" s="15" t="n"/>
+      <c r="G11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -4420,7 +4440,7 @@
         </is>
       </c>
       <c r="F12" s="16" t="n"/>
-      <c r="G12" s="15" t="n"/>
+      <c r="G12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -4449,7 +4469,7 @@
         </is>
       </c>
       <c r="F13" s="16" t="n"/>
-      <c r="G13" s="15" t="n"/>
+      <c r="G13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -4478,7 +4498,7 @@
         </is>
       </c>
       <c r="F14" s="16" t="n"/>
-      <c r="G14" s="15" t="n"/>
+      <c r="G14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -4507,7 +4527,7 @@
         </is>
       </c>
       <c r="F15" s="16" t="n"/>
-      <c r="G15" s="15" t="n"/>
+      <c r="G15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -4536,7 +4556,7 @@
         </is>
       </c>
       <c r="F16" s="16" t="n"/>
-      <c r="G16" s="15" t="n"/>
+      <c r="G16" s="17" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -4565,7 +4585,7 @@
         </is>
       </c>
       <c r="F17" s="16" t="n"/>
-      <c r="G17" s="15" t="n"/>
+      <c r="G17" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -4594,7 +4614,7 @@
         </is>
       </c>
       <c r="F18" s="16" t="n"/>
-      <c r="G18" s="15" t="n"/>
+      <c r="G18" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -4623,7 +4643,7 @@
         </is>
       </c>
       <c r="F19" s="16" t="n"/>
-      <c r="G19" s="15" t="n"/>
+      <c r="G19" s="17" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -4652,7 +4672,7 @@
         </is>
       </c>
       <c r="F20" s="16" t="n"/>
-      <c r="G20" s="15" t="n"/>
+      <c r="G20" s="17" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -4681,7 +4701,7 @@
         </is>
       </c>
       <c r="F21" s="16" t="n"/>
-      <c r="G21" s="15" t="n"/>
+      <c r="G21" s="17" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
@@ -4710,7 +4730,7 @@
         </is>
       </c>
       <c r="F22" s="16" t="n"/>
-      <c r="G22" s="15" t="n"/>
+      <c r="G22" s="17" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:G22"/>
@@ -4718,12 +4738,12 @@
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="2">
       <formula>"Discuss"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / Discuss" type="list">
+    <dataValidation sqref="F5:F22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / Discuss" type="list" errorStyle="stop">
       <formula1>"Yes,Discuss"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4809,7 +4829,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E5" s="15" t="n"/>
+      <c r="E5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -4832,7 +4852,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E6" s="15" t="n"/>
+      <c r="E6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -4855,7 +4875,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E7" s="15" t="n"/>
+      <c r="E7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -4878,7 +4898,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E8" s="15" t="n"/>
+      <c r="E8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4901,7 +4921,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E9" s="15" t="n"/>
+      <c r="E9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -4924,7 +4944,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E10" s="15" t="n"/>
+      <c r="E10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4947,7 +4967,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E11" s="15" t="n"/>
+      <c r="E11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -4970,7 +4990,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E12" s="15" t="n"/>
+      <c r="E12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -4993,7 +5013,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E13" s="15" t="n"/>
+      <c r="E13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -5016,7 +5036,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E14" s="15" t="n"/>
+      <c r="E14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -5039,7 +5059,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E15" s="15" t="n"/>
+      <c r="E15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -5062,7 +5082,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E16" s="15" t="n"/>
+      <c r="E16" s="17" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -5085,7 +5105,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E17" s="15" t="n"/>
+      <c r="E17" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -5108,7 +5128,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E18" s="15" t="n"/>
+      <c r="E18" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -5131,7 +5151,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E19" s="15" t="n"/>
+      <c r="E19" s="17" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -5154,7 +5174,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E20" s="15" t="n"/>
+      <c r="E20" s="17" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -5177,7 +5197,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E21" s="15" t="n"/>
+      <c r="E21" s="17" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
@@ -5200,7 +5220,7 @@
           <t>Not yet run</t>
         </is>
       </c>
-      <c r="E22" s="15" t="n"/>
+      <c r="E22" s="17" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:E22"/>
@@ -5219,7 +5239,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Pass / Fail / Deferred / Not yet run" type="list">
+    <dataValidation sqref="D5:D22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Pass / Fail / Deferred / Not yet run" type="list" errorStyle="stop">
       <formula1>"Pass,Fail,Deferred,Not yet run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5236,7 +5256,7 @@
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -5299,7 +5319,7 @@
         </is>
       </c>
       <c r="D5" s="16" t="n"/>
-      <c r="E5" s="15" t="n"/>
+      <c r="E5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="n">
@@ -5316,7 +5336,7 @@
         </is>
       </c>
       <c r="D6" s="16" t="n"/>
-      <c r="E6" s="15" t="n"/>
+      <c r="E6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="n">
@@ -5333,7 +5353,7 @@
         </is>
       </c>
       <c r="D7" s="16" t="n"/>
-      <c r="E7" s="15" t="n"/>
+      <c r="E7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="n">
@@ -5350,7 +5370,7 @@
         </is>
       </c>
       <c r="D8" s="16" t="n"/>
-      <c r="E8" s="15" t="n"/>
+      <c r="E8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="n">
@@ -5367,7 +5387,7 @@
         </is>
       </c>
       <c r="D9" s="16" t="n"/>
-      <c r="E9" s="15" t="n"/>
+      <c r="E9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="n">
@@ -5384,7 +5404,7 @@
         </is>
       </c>
       <c r="D10" s="16" t="n"/>
-      <c r="E10" s="15" t="n"/>
+      <c r="E10" s="17" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="n">
@@ -5401,7 +5421,7 @@
         </is>
       </c>
       <c r="D11" s="16" t="n"/>
-      <c r="E11" s="15" t="n"/>
+      <c r="E11" s="17" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="n">
@@ -5418,7 +5438,7 @@
         </is>
       </c>
       <c r="D12" s="16" t="n"/>
-      <c r="E12" s="15" t="n"/>
+      <c r="E12" s="17" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="12" t="n">
@@ -5435,7 +5455,7 @@
         </is>
       </c>
       <c r="D13" s="16" t="n"/>
-      <c r="E13" s="15" t="n"/>
+      <c r="E13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="n">
@@ -5452,7 +5472,7 @@
         </is>
       </c>
       <c r="D14" s="16" t="n"/>
-      <c r="E14" s="15" t="n"/>
+      <c r="E14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="n">
@@ -5469,7 +5489,7 @@
         </is>
       </c>
       <c r="D15" s="16" t="n"/>
-      <c r="E15" s="15" t="n"/>
+      <c r="E15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="n">
@@ -5486,7 +5506,7 @@
         </is>
       </c>
       <c r="D16" s="16" t="n"/>
-      <c r="E16" s="15" t="n"/>
+      <c r="E16" s="17" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12" t="n">
@@ -5503,7 +5523,7 @@
         </is>
       </c>
       <c r="D17" s="16" t="n"/>
-      <c r="E17" s="15" t="n"/>
+      <c r="E17" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="n">
@@ -5520,7 +5540,7 @@
         </is>
       </c>
       <c r="D18" s="16" t="n"/>
-      <c r="E18" s="15" t="n"/>
+      <c r="E18" s="17" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:E18"/>
@@ -5536,7 +5556,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / No / N/A" type="list">
+    <dataValidation sqref="D5:D18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / No / N/A" type="list" errorStyle="stop">
       <formula1>"Yes,No,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5550,7 +5570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5717,237 +5737,216 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Optional fifth (D12): Meditron-70B, dense, ~40 GB at 4-bit, single-digit tok/s, Minerva cross-check only, runs through llama.cpp in Phase 3 (C5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>The two hemispheres</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Ren Ackerman — Vanguard, Prime Director</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Arthur Sterling — Architect, Estate Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Hemisphere</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>Offensive, creative, expansive, outward-facing</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>Defensive, regimented, private, guardian of personal data</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Domain mandate</t>
+          <t>Hemisphere</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Corporate, Enterprise, Infrastructure, AEC</t>
+          <t>Offensive, creative, expansive, outward-facing</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Estate, Private Health, Logistics, Family</t>
+          <t>Defensive, regimented, private, guardian of personal data</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Default engine</t>
+          <t>Domain mandate</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>gpt-oss-120b</t>
+          <t>Corporate, Enterprise, Infrastructure, AEC</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Nemotron 3 Super</t>
+          <t>Estate, Private Health, Logistics, Family</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Override engine</t>
+          <t>Default engine</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>gpt-oss-120b abliterated, on Principal's order</t>
+          <t>gpt-oss-120b</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Qwen3.5-122B-A10B for deep document reasoning</t>
+          <t>Nemotron 3 Super</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Sampling</t>
+          <t>Override engine</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>High temperature (0.8) as Deep Think Generator</t>
+          <t>gpt-oss-120b abliterated, on Principal's order</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Low temperature, not zero, as Deep Think Adversary</t>
+          <t>Qwen3.5-122B-A10B for deep document reasoning</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Deep Think role</t>
+          <t>Sampling</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Generator: three divergent trajectories</t>
+          <t>High temperature (0.8) as Deep Think Generator</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Adversary: rubric-scored verdict, weak concepts killed</t>
+          <t>Low temperature, not zero, as Deep Think Adversary</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Code path</t>
+          <t>Deep Think role</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Writes sandbox code</t>
+          <t>Generator: three divergent trajectories</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Audits code for memory and safety before execution, as a second layer over the OS-level sandbox cap</t>
+          <t>Adversary: rubric-scored verdict, weak concepts killed</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
+          <t>Code path</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Writes sandbox code</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Audits code for memory and safety before execution, as a second layer over the OS-level sandbox cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
           <t>Directors</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Gideon, Silas, Valerie, Helena, Eleanor</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>Alaric, Minerva, Victor</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Shadow Cabinet engine map</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Director</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
         <is>
           <t>Remit</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>Default engine</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>Override</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
+      <c r="F24" s="10" t="inlineStr">
         <is>
           <t>Speaks externally</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>Gideon Vance</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>Corporate</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="inlineStr">
-        <is>
-          <t>Legal &amp; Compliance</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>gpt-oss-120b, high reasoning, retrieval-grounded</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>Qwen3.5-122B for long contracts</t>
-        </is>
-      </c>
-      <c r="F24" s="11" t="inlineStr">
-        <is>
-          <t>Yes, sensitive tier</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Silas Thorne</t>
+          <t>Gideon Vance</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
@@ -5957,29 +5956,29 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>CFO: capital, audit, banking</t>
+          <t>Legal &amp; Compliance</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Nemotron 3 Super + code interpreter for all arithmetic</t>
+          <t>gpt-oss-120b, high reasoning, retrieval-grounded</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Qwen3.5-122B for long contracts</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Yes, standard tier</t>
+          <t>Yes, sensitive tier</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Valerie Cross</t>
+          <t>Silas Thorne</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -5989,17 +5988,17 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Infrastructure, DevOps, AEC, cyber, AEGIS Sandbox</t>
+          <t>CFO: capital, audit, banking</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>gpt-oss-120b abliterated</t>
+          <t>Nemotron 3 Super + code interpreter for all arithmetic</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Qwen3.5-122B for drawings and images</t>
+          <t>none</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
@@ -6011,7 +6010,7 @@
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>Helena Frost</t>
+          <t>Valerie Cross</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
@@ -6021,17 +6020,17 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Communications, brand, PR, crisis</t>
+          <t>Infrastructure, DevOps, AEC, cyber, AEGIS Sandbox</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>gpt-oss-120b</t>
+          <t>gpt-oss-120b abliterated</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Qwen3.5-122B for drawings and images</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
@@ -6043,7 +6042,7 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Eleanor Croft</t>
+          <t>Helena Frost</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -6053,12 +6052,12 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Routing, scheduling, triage; the 4-Way Router's classifier</t>
+          <t>Communications, brand, PR, crisis</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Resident 4B model</t>
+          <t>gpt-oss-120b</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -6068,29 +6067,29 @@
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>Yes, routine tier (scheduling)</t>
+          <t>Yes, standard tier</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>Alaric Stone</t>
+          <t>Eleanor Croft</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Estate</t>
+          <t>Corporate</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Physical assets, security, threat mitigation; Sentinel threat watch</t>
+          <t>Routing, scheduling, triage; the 4-Way Router's classifier</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Nemotron 3 Super</t>
+          <t>Resident 4B model</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
@@ -6100,14 +6099,14 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Yes, sensitive tier</t>
+          <t>Yes, routine tier (scheduling)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Minerva Hale</t>
+          <t>Alaric Stone</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -6117,17 +6116,17 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Private health, longevity; medical data</t>
+          <t>Physical assets, security, threat mitigation; Sentinel threat watch</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>gpt-oss-120b, retrieval-grounded</t>
+          <t>Nemotron 3 Super</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Qwen3.5-122B for records and scans; Meditron-70B cross-check</t>
+          <t>none</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -6139,30 +6138,62 @@
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
+          <t>Minerva Hale</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Estate</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Private health, longevity; medical data</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>gpt-oss-120b, retrieval-grounded</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Qwen3.5-122B for records and scans; Meditron-70B cross-check</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Yes, sensitive tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
           <t>Victor Vale</t>
         </is>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Estate</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>Aviation, transport, concierge</t>
         </is>
       </c>
-      <c r="D31" s="11" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>gpt-oss-120b</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr">
+      <c r="F32" s="11" t="inlineStr">
         <is>
           <t>Yes, routine tier</t>
         </is>

</xml_diff>

<commit_message>
Tighten legend wording in the confirmation workbook
Legend and mapping note now list the exact dropdown values, state that
"Not yet run" counts as Remaining, and explain the Verification sheet's
amber pre-fill.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USyWZdFCwDpe3L4dpdaCcG
</commit_message>
<xml_diff>
--- a/docs/ATLAS_REVIEW_CONFIRMATION.xlsx
+++ b/docs/ATLAS_REVIEW_CONFIRMATION.xlsx
@@ -615,7 +615,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>4. Sheet 4 (Verification) is filled during Day 1 as each phase gate runs, not now.</t>
+          <t>4. Sheet 4 (Verification) is filled during Day 1 as each phase gate runs, not now; its Result column shows amber 'Not yet run' until then.</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Need more information / Deferred / Not yet run</t>
+          <t>Need more information / Deferred / Not yet run (Not yet run counts as Remaining, not Hold)</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Change / Disagree / Discuss / No / Fail</t>
+          <t>Change / Disagree - return to decisions / Discuss / No / Fail</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Positive / Hold / Negative map to each sheet's dropdown: Decisions = Accept / Need more information / Change; Resolutions = Accept / - / Disagree; Risks = Yes / - / Discuss; Verification = Pass / Deferred / Fail; Checklist = Yes or N/A / - / No.</t>
+          <t>Positive / Hold / Negative map to each sheet's dropdown: Decisions = Accept / Need more information / Change; Resolutions = Accept / - / Disagree - return to decisions; Risks = Yes / - / Discuss; Verification = Pass / Deferred / Fail, with Not yet run counted as Remaining; Checklist = Yes or N/A / - / No.</t>
         </is>
       </c>
     </row>

</xml_diff>